<commit_message>
L7 其他非流动负债真双向（五环发布+模板净化+manifest翻bidirectional+真OO往返）：task76 五环 provision + first_publication representation gen1 DB 三表闭环（bundle approved）；受管表 明细表L7-2 横向共享公式组 M12:N16 净化展开（受管 sheet 0 diff，sha 9fe0→35e4）；overlay 补 L7 override + 干净 worktree 重算 approved_source_digest 7ae8f4c7，mount-diff 零能力损失唯一翻转 L7；真 OO 引擎往返 9 步全绿（公式 E/L/M/N/O 幸存+rowId 稳定无幽灵行+不写库）
</commit_message>
<xml_diff>
--- a/backend/wp_templates/L/L7 其他非流动负债.xlsx
+++ b/backend/wp_templates/L/L7 其他非流动负债.xlsx
@@ -6461,11 +6461,11 @@
         <v>0</v>
       </c>
       <c r="M12" s="86">
-        <f t="shared" ref="M12:N16" si="0">C12+H12+J12</f>
+        <f>C12+H12+J12</f>
         <v>0</v>
       </c>
       <c r="N12" s="86">
-        <f t="shared" si="0"/>
+        <f>D12+I12+K12</f>
         <v>0</v>
       </c>
       <c r="O12" s="86">
@@ -6496,15 +6496,15 @@
         <v>0</v>
       </c>
       <c r="M13" s="86">
-        <f t="shared" si="0"/>
+        <f>C13+H13+J13</f>
         <v>0</v>
       </c>
       <c r="N13" s="86">
-        <f t="shared" si="0"/>
+        <f>D13+I13+K13</f>
         <v>0</v>
       </c>
       <c r="O13" s="86">
-        <f t="shared" ref="O13:O16" si="1">L13+M13-N13</f>
+        <f>L13+M13-N13</f>
         <v>0</v>
       </c>
       <c r="P13" s="95"/>
@@ -6531,15 +6531,15 @@
         <v>0</v>
       </c>
       <c r="M14" s="86">
-        <f t="shared" si="0"/>
+        <f>C14+H14+J14</f>
         <v>0</v>
       </c>
       <c r="N14" s="86">
-        <f t="shared" si="0"/>
+        <f>D14+I14+K14</f>
         <v>0</v>
       </c>
       <c r="O14" s="86">
-        <f t="shared" si="1"/>
+        <f>L14+M14-N14</f>
         <v>0</v>
       </c>
       <c r="P14" s="95"/>
@@ -6566,15 +6566,15 @@
         <v>0</v>
       </c>
       <c r="M15" s="86">
-        <f t="shared" si="0"/>
+        <f>C15+H15+J15</f>
         <v>0</v>
       </c>
       <c r="N15" s="86">
-        <f t="shared" si="0"/>
+        <f>D15+I15+K15</f>
         <v>0</v>
       </c>
       <c r="O15" s="86">
-        <f t="shared" si="1"/>
+        <f>L15+M15-N15</f>
         <v>0</v>
       </c>
       <c r="P15" s="95"/>
@@ -6601,15 +6601,15 @@
         <v>0</v>
       </c>
       <c r="M16" s="86">
-        <f t="shared" si="0"/>
+        <f>C16+H16+J16</f>
         <v>0</v>
       </c>
       <c r="N16" s="86">
-        <f t="shared" si="0"/>
+        <f>D16+I16+K16</f>
         <v>0</v>
       </c>
       <c r="O16" s="86">
-        <f t="shared" si="1"/>
+        <f>L16+M16-N16</f>
         <v>0</v>
       </c>
       <c r="P16" s="95"/>
@@ -6621,59 +6621,59 @@
         <v>84</v>
       </c>
       <c r="B17" s="86">
-        <f t="shared" ref="B17:O17" si="2">SUM(B12:B16)</f>
+        <f>SUM(B12:B16)</f>
         <v>0</v>
       </c>
       <c r="C17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(C12:C16)</f>
         <v>0</v>
       </c>
       <c r="D17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(D12:D16)</f>
         <v>0</v>
       </c>
       <c r="E17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(E12:E16)</f>
         <v>0</v>
       </c>
       <c r="F17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(F12:F16)</f>
         <v>0</v>
       </c>
       <c r="G17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(G12:G16)</f>
         <v>0</v>
       </c>
       <c r="H17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(H12:H16)</f>
         <v>0</v>
       </c>
       <c r="I17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(I12:I16)</f>
         <v>0</v>
       </c>
       <c r="J17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(J12:J16)</f>
         <v>0</v>
       </c>
       <c r="K17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(K12:K16)</f>
         <v>0</v>
       </c>
       <c r="L17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(L12:L16)</f>
         <v>0</v>
       </c>
       <c r="M17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(M12:M16)</f>
         <v>0</v>
       </c>
       <c r="N17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(N12:N16)</f>
         <v>0</v>
       </c>
       <c r="O17" s="86">
-        <f t="shared" si="2"/>
+        <f>SUM(O12:O16)</f>
         <v>0</v>
       </c>
       <c r="P17" s="179"/>

</xml_diff>